<commit_message>
fix: use system git credential instead of runtime secret for Windows clone
Woodpecker blocks secret injection for non-allowlisted clone images, so
FORGEJO_TOKEN was never populated and the clone fell back to GCM (which
needs an interactive OAuth TTY that CI doesn't have).

Fix: deploy-windows-agent.ps1 now stores the Forgejo PAT as a git system-
level http.extraHeader for git.cbp-org.internal and disables GCM for that
host. Git authenticates silently as any user (including SYSTEM) without
needing runtime secrets in the pipeline.

verify-windows.yml no longer needs a custom clone step or any clone
secrets — the standard Woodpecker local-backend clone just works.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/samples/reports/sample_data_large/types/Improvement.xlsx
+++ b/data/samples/reports/sample_data_large/types/Improvement.xlsx
@@ -2655,7 +2655,7 @@
       <c r="J36" s="0"/>
       <c r="K36" s="0"/>
       <c r="L36" s="0" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="M36" s="0"/>
       <c r="N36" s="0"/>
@@ -3023,7 +3023,7 @@
       <c r="J42" s="0"/>
       <c r="K42" s="0"/>
       <c r="L42" s="0" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="M42" s="0"/>
       <c r="N42" s="0"/>
@@ -3066,7 +3066,7 @@
       <c r="J43" s="0"/>
       <c r="K43" s="0"/>
       <c r="L43" s="0" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="M43" s="0"/>
       <c r="N43" s="0"/>
@@ -3109,7 +3109,7 @@
       <c r="J44" s="0"/>
       <c r="K44" s="0"/>
       <c r="L44" s="0" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M44" s="0"/>
       <c r="N44" s="0"/>
@@ -3152,7 +3152,7 @@
       <c r="J45" s="0"/>
       <c r="K45" s="0"/>
       <c r="L45" s="0" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M45" s="0"/>
       <c r="N45" s="0"/>
@@ -3195,7 +3195,7 @@
       <c r="J46" s="0"/>
       <c r="K46" s="0"/>
       <c r="L46" s="0" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="M46" s="0"/>
       <c r="N46" s="0"/>
@@ -3238,7 +3238,7 @@
       <c r="J47" s="0"/>
       <c r="K47" s="0"/>
       <c r="L47" s="0" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="M47" s="0"/>
       <c r="N47" s="0"/>
@@ -3281,7 +3281,7 @@
       <c r="J48" s="0"/>
       <c r="K48" s="0"/>
       <c r="L48" s="0" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M48" s="0"/>
       <c r="N48" s="0"/>
@@ -3324,7 +3324,7 @@
       <c r="J49" s="0"/>
       <c r="K49" s="0"/>
       <c r="L49" s="0" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M49" s="0"/>
       <c r="N49" s="0"/>
@@ -3367,7 +3367,7 @@
       <c r="J50" s="0"/>
       <c r="K50" s="0"/>
       <c r="L50" s="0" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="M50" s="0"/>
       <c r="N50" s="0"/>
@@ -3410,7 +3410,7 @@
       <c r="J51" s="0"/>
       <c r="K51" s="0"/>
       <c r="L51" s="0" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="M51" s="0"/>
       <c r="N51" s="0"/>

</xml_diff>